<commit_message>
vault backup: 2026-04-28 10:14:46
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/PEP/Model Output/PEP_model_v10.xlsx
+++ b/Knowledge/Model Schema/PEP/Model Output/PEP_model_v10.xlsx
@@ -7475,79 +7475,79 @@
         <v/>
       </c>
       <c r="S46" s="12">
-        <f>S25+S33+S44+S45+S46</f>
+        <f>S25+S33+S44+S45</f>
         <v/>
       </c>
       <c r="T46" s="12">
-        <f>T25+T33+T44+T45+T46</f>
+        <f>T25+T33+T44+T45</f>
         <v/>
       </c>
       <c r="U46" s="12">
-        <f>U25+U33+U44+U45+U46</f>
+        <f>U25+U33+U44+U45</f>
         <v/>
       </c>
       <c r="V46" s="12">
-        <f>V25+V33+V44+V45+V46</f>
+        <f>V25+V33+V44+V45</f>
         <v/>
       </c>
       <c r="W46" s="12">
-        <f>W25+W33+W44+W45+W46</f>
+        <f>W25+W33+W44+W45</f>
         <v/>
       </c>
       <c r="X46" s="12">
-        <f>X25+X33+X44+X45+X46</f>
+        <f>X25+X33+X44+X45</f>
         <v/>
       </c>
       <c r="Y46" s="12">
-        <f>Y25+Y33+Y44+Y45+Y46</f>
+        <f>Y25+Y33+Y44+Y45</f>
         <v/>
       </c>
       <c r="Z46" s="12">
-        <f>Z25+Z33+Z44+Z45+Z46</f>
+        <f>Z25+Z33+Z44+Z45</f>
         <v/>
       </c>
       <c r="AA46" s="12">
-        <f>AA25+AA33+AA44+AA45+AA46</f>
+        <f>AA25+AA33+AA44+AA45</f>
         <v/>
       </c>
       <c r="AB46" s="12">
-        <f>AB25+AB33+AB44+AB45+AB46</f>
+        <f>AB25+AB33+AB44+AB45</f>
         <v/>
       </c>
       <c r="AC46" s="12">
-        <f>AC25+AC33+AC44+AC45+AC46</f>
+        <f>AC25+AC33+AC44+AC45</f>
         <v/>
       </c>
       <c r="AD46" s="12">
-        <f>AD25+AD33+AD44+AD45+AD46</f>
+        <f>AD25+AD33+AD44+AD45</f>
         <v/>
       </c>
       <c r="AE46" s="12">
-        <f>AE25+AE33+AE44+AE45+AE46</f>
+        <f>AE25+AE33+AE44+AE45</f>
         <v/>
       </c>
       <c r="AF46" s="12">
-        <f>AF25+AF33+AF44+AF45+AF46</f>
+        <f>AF25+AF33+AF44+AF45</f>
         <v/>
       </c>
       <c r="AG46" s="12">
-        <f>AG25+AG33+AG44+AG45+AG46</f>
+        <f>AG25+AG33+AG44+AG45</f>
         <v/>
       </c>
       <c r="AH46" s="12">
-        <f>AH25+AH33+AH44+AH45+AH46</f>
+        <f>AH25+AH33+AH44+AH45</f>
         <v/>
       </c>
       <c r="AI46" s="12">
-        <f>AI25+AI33+AI44+AI45+AI46</f>
+        <f>AI25+AI33+AI44+AI45</f>
         <v/>
       </c>
       <c r="AJ46" s="12">
-        <f>AJ25+AJ33+AJ44+AJ45+AJ46</f>
+        <f>AJ25+AJ33+AJ44+AJ45</f>
         <v/>
       </c>
       <c r="AK46" s="12">
-        <f>AK25+AK33+AK44+AK45+AK46</f>
+        <f>AK25+AK33+AK44+AK45</f>
         <v/>
       </c>
     </row>
@@ -22638,47 +22638,47 @@
         </is>
       </c>
       <c r="B48" s="6">
-        <f>B26+B34+B46+B47+B48</f>
+        <f>B26+B34+B46+B47</f>
         <v/>
       </c>
       <c r="C48" s="6">
-        <f>C26+C34+C46+C47+C48</f>
+        <f>C26+C34+C46+C47</f>
         <v/>
       </c>
       <c r="D48" s="6">
-        <f>D26+D34+D46+D47+D48</f>
+        <f>D26+D34+D46+D47</f>
         <v/>
       </c>
       <c r="E48" s="6">
-        <f>E26+E34+E46+E47+E48</f>
+        <f>E26+E34+E46+E47</f>
         <v/>
       </c>
       <c r="F48" s="6">
-        <f>F26+F34+F46+F47+F48</f>
+        <f>F26+F34+F46+F47</f>
         <v/>
       </c>
       <c r="G48" s="7">
-        <f>G26+G34+G46+G47+G48</f>
+        <f>G26+G34+G46+G47</f>
         <v/>
       </c>
       <c r="H48" s="7">
-        <f>H26+H34+H46+H47+H48</f>
+        <f>H26+H34+H46+H47</f>
         <v/>
       </c>
       <c r="I48" s="7">
-        <f>I26+I34+I46+I47+I48</f>
+        <f>I26+I34+I46+I47</f>
         <v/>
       </c>
       <c r="J48" s="7">
-        <f>J26+J34+J46+J47+J48</f>
+        <f>J26+J34+J46+J47</f>
         <v/>
       </c>
       <c r="K48" s="7">
-        <f>K26+K34+K46+K47+K48</f>
+        <f>K26+K34+K46+K47</f>
         <v/>
       </c>
       <c r="L48" s="7">
-        <f>L26+L34+L46+L47+L48</f>
+        <f>L26+L34+L46+L47</f>
         <v/>
       </c>
     </row>
@@ -27401,55 +27401,55 @@
         </is>
       </c>
       <c r="B46" s="6">
-        <f>B25+B33+B44+B45+B46</f>
+        <f>B25+B33+B44+B45</f>
         <v/>
       </c>
       <c r="C46" s="6">
-        <f>C25+C33+C44+C45+C46</f>
+        <f>C25+C33+C44+C45</f>
         <v/>
       </c>
       <c r="D46" s="6">
-        <f>D25+D33+D44+D45+D46</f>
+        <f>D25+D33+D44+D45</f>
         <v/>
       </c>
       <c r="E46" s="6">
-        <f>E25+E33+E44+E45+E46</f>
+        <f>E25+E33+E44+E45</f>
         <v/>
       </c>
       <c r="F46" s="6">
-        <f>F25+F33+F44+F45+F46</f>
+        <f>F25+F33+F44+F45</f>
         <v/>
       </c>
       <c r="G46" s="6">
-        <f>G25+G33+G44+G45+G46</f>
+        <f>G25+G33+G44+G45</f>
         <v/>
       </c>
       <c r="H46" s="6">
-        <f>H25+H33+H44+H45+H46</f>
+        <f>H25+H33+H44+H45</f>
         <v/>
       </c>
       <c r="I46" s="6">
-        <f>I25+I33+I44+I45+I46</f>
+        <f>I25+I33+I44+I45</f>
         <v/>
       </c>
       <c r="J46" s="6">
-        <f>J25+J33+J44+J45+J46</f>
+        <f>J25+J33+J44+J45</f>
         <v/>
       </c>
       <c r="K46" s="6">
-        <f>K25+K33+K44+K45+K46</f>
+        <f>K25+K33+K44+K45</f>
         <v/>
       </c>
       <c r="L46" s="6">
-        <f>L25+L33+L44+L45+L46</f>
+        <f>L25+L33+L44+L45</f>
         <v/>
       </c>
       <c r="M46" s="6">
-        <f>M25+M33+M44+M45+M46</f>
+        <f>M25+M33+M44+M45</f>
         <v/>
       </c>
       <c r="N46" s="6">
-        <f>N25+N33+N44+N45+N46</f>
+        <f>N25+N33+N44+N45</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-04-28 10:19:56
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/PEP/Model Output/PEP_model_v10.xlsx
+++ b/Knowledge/Model Schema/PEP/Model Output/PEP_model_v10.xlsx
@@ -11762,80 +11762,80 @@
         <f>'QTR BS'!O23</f>
         <v/>
       </c>
-      <c r="P19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="Q19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="R19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="S19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="T19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="U19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="V19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="W19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="X19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="Y19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="Z19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="AA19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="AB19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="AC19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="AD19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="AE19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="AF19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="AG19" s="15">
-        <f>O19</f>
-        <v/>
-      </c>
-      <c r="AH19" s="15">
-        <f>O19</f>
+      <c r="P19" s="4">
+        <f>O19+'QTR CF'!S9</f>
+        <v/>
+      </c>
+      <c r="Q19" s="4">
+        <f>P19+'QTR CF'!T9</f>
+        <v/>
+      </c>
+      <c r="R19" s="4">
+        <f>Q19+'QTR CF'!U9</f>
+        <v/>
+      </c>
+      <c r="S19" s="4">
+        <f>R19+'QTR CF'!V9</f>
+        <v/>
+      </c>
+      <c r="T19" s="4">
+        <f>S19+'QTR CF'!W9</f>
+        <v/>
+      </c>
+      <c r="U19" s="4">
+        <f>T19+'QTR CF'!X9</f>
+        <v/>
+      </c>
+      <c r="V19" s="4">
+        <f>U19+'QTR CF'!Y9</f>
+        <v/>
+      </c>
+      <c r="W19" s="4">
+        <f>V19+'QTR CF'!Z9</f>
+        <v/>
+      </c>
+      <c r="X19" s="4">
+        <f>W19+'QTR CF'!AA9</f>
+        <v/>
+      </c>
+      <c r="Y19" s="4">
+        <f>X19+'QTR CF'!AB9</f>
+        <v/>
+      </c>
+      <c r="Z19" s="4">
+        <f>Y19+'QTR CF'!AC9</f>
+        <v/>
+      </c>
+      <c r="AA19" s="4">
+        <f>Z19+'QTR CF'!AD9</f>
+        <v/>
+      </c>
+      <c r="AB19" s="4">
+        <f>AA19+'QTR CF'!AE9</f>
+        <v/>
+      </c>
+      <c r="AC19" s="4">
+        <f>AB19+'QTR CF'!AF9</f>
+        <v/>
+      </c>
+      <c r="AD19" s="4">
+        <f>AC19+'QTR CF'!AG9</f>
+        <v/>
+      </c>
+      <c r="AE19" s="4">
+        <f>AD19+'QTR CF'!AH9</f>
+        <v/>
+      </c>
+      <c r="AF19" s="4">
+        <f>AE19+'QTR CF'!AI9</f>
+        <v/>
+      </c>
+      <c r="AG19" s="4">
+        <f>AF19+'QTR CF'!AJ9</f>
+        <v/>
+      </c>
+      <c r="AH19" s="4">
+        <f>AG19+'QTR CF'!AK9</f>
         <v/>
       </c>
     </row>
@@ -12040,80 +12040,80 @@
         <f>'QTR BS'!O25</f>
         <v/>
       </c>
-      <c r="P21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="Q21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="R21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="S21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="T21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="U21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="V21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="W21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="X21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="Y21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="Z21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="AA21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="AB21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="AC21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="AD21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="AE21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="AF21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="AG21" s="15">
-        <f>O21</f>
-        <v/>
-      </c>
-      <c r="AH21" s="15">
-        <f>O21</f>
+      <c r="P21" s="4">
+        <f>O21+'QTR CF'!S45</f>
+        <v/>
+      </c>
+      <c r="Q21" s="4">
+        <f>P21+'QTR CF'!T45</f>
+        <v/>
+      </c>
+      <c r="R21" s="4">
+        <f>Q21+'QTR CF'!U45</f>
+        <v/>
+      </c>
+      <c r="S21" s="4">
+        <f>R21+'QTR CF'!V45</f>
+        <v/>
+      </c>
+      <c r="T21" s="4">
+        <f>S21+'QTR CF'!W45</f>
+        <v/>
+      </c>
+      <c r="U21" s="4">
+        <f>T21+'QTR CF'!X45</f>
+        <v/>
+      </c>
+      <c r="V21" s="4">
+        <f>U21+'QTR CF'!Y45</f>
+        <v/>
+      </c>
+      <c r="W21" s="4">
+        <f>V21+'QTR CF'!Z45</f>
+        <v/>
+      </c>
+      <c r="X21" s="4">
+        <f>W21+'QTR CF'!AA45</f>
+        <v/>
+      </c>
+      <c r="Y21" s="4">
+        <f>X21+'QTR CF'!AB45</f>
+        <v/>
+      </c>
+      <c r="Z21" s="4">
+        <f>Y21+'QTR CF'!AC45</f>
+        <v/>
+      </c>
+      <c r="AA21" s="4">
+        <f>Z21+'QTR CF'!AD45</f>
+        <v/>
+      </c>
+      <c r="AB21" s="4">
+        <f>AA21+'QTR CF'!AE45</f>
+        <v/>
+      </c>
+      <c r="AC21" s="4">
+        <f>AB21+'QTR CF'!AF45</f>
+        <v/>
+      </c>
+      <c r="AD21" s="4">
+        <f>AC21+'QTR CF'!AG45</f>
+        <v/>
+      </c>
+      <c r="AE21" s="4">
+        <f>AD21+'QTR CF'!AH45</f>
+        <v/>
+      </c>
+      <c r="AF21" s="4">
+        <f>AE21+'QTR CF'!AI45</f>
+        <v/>
+      </c>
+      <c r="AG21" s="4">
+        <f>AF21+'QTR CF'!AJ45</f>
+        <v/>
+      </c>
+      <c r="AH21" s="4">
+        <f>AG21+'QTR CF'!AK45</f>
         <v/>
       </c>
     </row>
@@ -14633,62 +14633,81 @@
         <f>'QTR CF'!R16</f>
         <v/>
       </c>
-      <c r="S16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="U16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="V16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="W16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="X16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK16" s="15" t="n">
-        <v>0</v>
+      <c r="S16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="T16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="U16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="V16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="W16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="X16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="Y16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="Z16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AA16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AB16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AC16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AD16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AE16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AF16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AG16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AH16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AI16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AJ16" s="15">
+        <f>R16</f>
+        <v/>
+      </c>
+      <c r="AK16" s="15">
+        <f>R16</f>
+        <v/>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
vault backup: 2026-04-28 10:25:07
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/PEP/Model Output/PEP_model_v10.xlsx
+++ b/Knowledge/Model Schema/PEP/Model Output/PEP_model_v10.xlsx
@@ -1737,79 +1737,79 @@
         <v/>
       </c>
       <c r="S8" s="11">
-        <f>'QTR P&amp;L'!S2*'CF DRIVERS'!S8</f>
+        <f>'CF DRIVERS'!S8</f>
         <v/>
       </c>
       <c r="T8" s="11">
-        <f>'QTR P&amp;L'!T2*'CF DRIVERS'!T8</f>
+        <f>'CF DRIVERS'!T8</f>
         <v/>
       </c>
       <c r="U8" s="11">
-        <f>'QTR P&amp;L'!U2*'CF DRIVERS'!U8</f>
+        <f>'CF DRIVERS'!U8</f>
         <v/>
       </c>
       <c r="V8" s="11">
-        <f>'QTR P&amp;L'!V2*'CF DRIVERS'!V8</f>
+        <f>'CF DRIVERS'!V8</f>
         <v/>
       </c>
       <c r="W8" s="11">
-        <f>'QTR P&amp;L'!W2*'CF DRIVERS'!W8</f>
+        <f>'CF DRIVERS'!W8</f>
         <v/>
       </c>
       <c r="X8" s="11">
-        <f>'QTR P&amp;L'!X2*'CF DRIVERS'!X8</f>
+        <f>'CF DRIVERS'!X8</f>
         <v/>
       </c>
       <c r="Y8" s="11">
-        <f>'QTR P&amp;L'!Y2*'CF DRIVERS'!Y8</f>
+        <f>'CF DRIVERS'!Y8</f>
         <v/>
       </c>
       <c r="Z8" s="11">
-        <f>'QTR P&amp;L'!Z2*'CF DRIVERS'!Z8</f>
+        <f>'CF DRIVERS'!Z8</f>
         <v/>
       </c>
       <c r="AA8" s="11">
-        <f>'QTR P&amp;L'!AA2*'CF DRIVERS'!AA8</f>
+        <f>'CF DRIVERS'!AA8</f>
         <v/>
       </c>
       <c r="AB8" s="11">
-        <f>'QTR P&amp;L'!AB2*'CF DRIVERS'!AB8</f>
+        <f>'CF DRIVERS'!AB8</f>
         <v/>
       </c>
       <c r="AC8" s="11">
-        <f>'QTR P&amp;L'!AC2*'CF DRIVERS'!AC8</f>
+        <f>'CF DRIVERS'!AC8</f>
         <v/>
       </c>
       <c r="AD8" s="11">
-        <f>'QTR P&amp;L'!AD2*'CF DRIVERS'!AD8</f>
+        <f>'CF DRIVERS'!AD8</f>
         <v/>
       </c>
       <c r="AE8" s="11">
-        <f>'QTR P&amp;L'!AE2*'CF DRIVERS'!AE8</f>
+        <f>'CF DRIVERS'!AE8</f>
         <v/>
       </c>
       <c r="AF8" s="11">
-        <f>'QTR P&amp;L'!AF2*'CF DRIVERS'!AF8</f>
+        <f>'CF DRIVERS'!AF8</f>
         <v/>
       </c>
       <c r="AG8" s="11">
-        <f>'QTR P&amp;L'!AG2*'CF DRIVERS'!AG8</f>
+        <f>'CF DRIVERS'!AG8</f>
         <v/>
       </c>
       <c r="AH8" s="11">
-        <f>'QTR P&amp;L'!AH2*'CF DRIVERS'!AH8</f>
+        <f>'CF DRIVERS'!AH8</f>
         <v/>
       </c>
       <c r="AI8" s="11">
-        <f>'QTR P&amp;L'!AI2*'CF DRIVERS'!AI8</f>
+        <f>'CF DRIVERS'!AI8</f>
         <v/>
       </c>
       <c r="AJ8" s="11">
-        <f>'QTR P&amp;L'!AJ2*'CF DRIVERS'!AJ8</f>
+        <f>'CF DRIVERS'!AJ8</f>
         <v/>
       </c>
       <c r="AK8" s="11">
-        <f>'QTR P&amp;L'!AK2*'CF DRIVERS'!AK8</f>
+        <f>'CF DRIVERS'!AK8</f>
         <v/>
       </c>
     </row>
@@ -13468,152 +13468,133 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Operating Lease ROU Asset Amortization — % of Revenue</t>
-        </is>
-      </c>
-      <c r="B8" s="13">
-        <f>IFERROR('QTR CF'!B8/'QTR P&amp;L'!B2,"")</f>
-        <v/>
-      </c>
-      <c r="C8" s="13">
-        <f>IFERROR('QTR CF'!C8/'QTR P&amp;L'!C2,"")</f>
-        <v/>
-      </c>
-      <c r="D8" s="13">
-        <f>IFERROR('QTR CF'!D8/'QTR P&amp;L'!D2,"")</f>
-        <v/>
-      </c>
-      <c r="E8" s="13">
-        <f>IFERROR('QTR CF'!E8/'QTR P&amp;L'!E2,"")</f>
-        <v/>
-      </c>
-      <c r="F8" s="13">
-        <f>IFERROR('QTR CF'!F8/'QTR P&amp;L'!F2,"")</f>
-        <v/>
-      </c>
-      <c r="G8" s="13">
-        <f>IFERROR('QTR CF'!G8/'QTR P&amp;L'!G2,"")</f>
-        <v/>
-      </c>
-      <c r="H8" s="13">
-        <f>IFERROR('QTR CF'!H8/'QTR P&amp;L'!H2,"")</f>
-        <v/>
-      </c>
-      <c r="I8" s="13">
-        <f>IFERROR('QTR CF'!I8/'QTR P&amp;L'!I2,"")</f>
-        <v/>
-      </c>
-      <c r="J8" s="13">
-        <f>IFERROR('QTR CF'!J8/'QTR P&amp;L'!J2,"")</f>
-        <v/>
-      </c>
-      <c r="K8" s="13">
-        <f>IFERROR('QTR CF'!K8/'QTR P&amp;L'!K2,"")</f>
-        <v/>
-      </c>
-      <c r="L8" s="13">
-        <f>IFERROR('QTR CF'!L8/'QTR P&amp;L'!L2,"")</f>
-        <v/>
-      </c>
-      <c r="M8" s="13">
-        <f>IFERROR('QTR CF'!M8/'QTR P&amp;L'!M2,"")</f>
-        <v/>
-      </c>
-      <c r="N8" s="13">
-        <f>IFERROR('QTR CF'!N8/'QTR P&amp;L'!N2,"")</f>
-        <v/>
-      </c>
-      <c r="O8" s="13">
-        <f>IFERROR('QTR CF'!O8/'QTR P&amp;L'!O2,"")</f>
-        <v/>
-      </c>
-      <c r="P8" s="13">
-        <f>IFERROR('QTR CF'!P8/'QTR P&amp;L'!P2,"")</f>
-        <v/>
-      </c>
-      <c r="Q8" s="13">
-        <f>IFERROR('QTR CF'!Q8/'QTR P&amp;L'!Q2,"")</f>
-        <v/>
-      </c>
-      <c r="R8" s="13">
-        <f>IFERROR('QTR CF'!R8/'QTR P&amp;L'!R2,"")</f>
-        <v/>
-      </c>
-      <c r="S8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="T8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="U8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="V8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="W8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="X8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="Y8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="Z8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AA8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AB8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AC8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AD8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AE8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AF8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AG8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AH8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AI8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AJ8" s="14">
-        <f>R8</f>
-        <v/>
-      </c>
-      <c r="AK8" s="14">
-        <f>R8</f>
-        <v/>
+          <t>Operating Lease ROU Asset Amortization</t>
+        </is>
+      </c>
+      <c r="B8" s="4">
+        <f>'QTR CF'!B8</f>
+        <v/>
+      </c>
+      <c r="C8" s="4">
+        <f>'QTR CF'!C8</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>'QTR CF'!D8</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>'QTR CF'!E8</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>'QTR CF'!F8</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>'QTR CF'!G8</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>'QTR CF'!H8</f>
+        <v/>
+      </c>
+      <c r="I8" s="4">
+        <f>'QTR CF'!I8</f>
+        <v/>
+      </c>
+      <c r="J8" s="4">
+        <f>'QTR CF'!J8</f>
+        <v/>
+      </c>
+      <c r="K8" s="4">
+        <f>'QTR CF'!K8</f>
+        <v/>
+      </c>
+      <c r="L8" s="4">
+        <f>'QTR CF'!L8</f>
+        <v/>
+      </c>
+      <c r="M8" s="4">
+        <f>'QTR CF'!M8</f>
+        <v/>
+      </c>
+      <c r="N8" s="4">
+        <f>'QTR CF'!N8</f>
+        <v/>
+      </c>
+      <c r="O8" s="4">
+        <f>'QTR CF'!O8</f>
+        <v/>
+      </c>
+      <c r="P8" s="4">
+        <f>'QTR CF'!P8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="4">
+        <f>'QTR CF'!Q8</f>
+        <v/>
+      </c>
+      <c r="R8" s="4">
+        <f>'QTR CF'!R8</f>
+        <v/>
+      </c>
+      <c r="S8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">

</xml_diff>